<commit_message>
Add 2024-vs-2026 comparison to deck and workbook
- Deck: two new slides — full CAPEX from 2024 feasibility study ($40.7M)
  and 2024->2026 equipment package comparison with deltas (now 11 slides)
- Workbook: CAPEX_2024 sheet and Сравнение_2024_2026 sheet with live
  delta formulas (now 8 sheets)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HURhMbsdrsD6qLQusHMshv
</commit_message>
<xml_diff>
--- a/Kazbiofert_Budget.xlsx
+++ b/Kazbiofert_Budget.xlsx
@@ -13,6 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="КИПиА" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Клапаны" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Электромонтаж" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX_2024" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сравнение_2024_2026" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,11 +23,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;"/>
+    <numFmt numFmtId="166" formatCode="+0%;-0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +80,12 @@
       <i val="1"/>
       <color rgb="00B57B00"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B57B00"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -133,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -214,6 +223,27 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1689,4 +1719,340 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Полный CAPEX по ТЭО (Kusto Chimkent, 23.07.2024) — USD, без НДС</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Тот же проект (Sairam / Kazbiofert). Файлы 2026 обновляют только оборудование внутри этого CAPEX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Проектные работы (Design)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>1124000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Биогазовый завод</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>15124611.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Завод твёрдых удобрений</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>11821211.71</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Preliminaries (мобилизация, персонал, техника)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>2358200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>— Подытог (основные разделы)</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="n">
+        <v>30428023.52</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Прочие объекты (офис, охрана, общежитие, лагуна, ОСВ, склад, благоустройство)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>6052005.93</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>— Подытог</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="n">
+        <v>36480029.45</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Накладные и прибыль ГенПодрядчика (~11,6%)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>4242723.53</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>ГРАНД-ИТОГО (без НДС)</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>40722752.98</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>в т.ч. строительная часть (Civil Works)</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="n">
+        <v>16568625.51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Сравнение: ТЭО 2024 → прайсы 2026 (пакет «железа», ≈USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Пакет</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2024, USD</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>2026, ≈USD</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Δ, USD</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Δ, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>Технологическое оборудование</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="n">
+        <v>10450000</v>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>12160982</v>
+      </c>
+      <c r="D4" s="23">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="33">
+        <f>C4/B4-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Клапаны / арматура</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>174120</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>310104</v>
+      </c>
+      <c r="D5" s="7">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="34">
+        <f>C5/B5-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>КИПиА (приборы)</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>66342</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>561705</v>
+      </c>
+      <c r="D6" s="23">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="33">
+        <f>C6/B6-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Трубопроводы, трафо, СН/ВН (нет в 2026)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>1360000</v>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Сравнимый пакет (обор.+клапаны+КИП)</t>
+        </is>
+      </c>
+      <c r="B8" s="16">
+        <f>SUM(B4:B6)</f>
+        <v/>
+      </c>
+      <c r="C8" s="16">
+        <f>SUM(C4:C6)</f>
+        <v/>
+      </c>
+      <c r="D8" s="16">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="36">
+        <f>C8/B8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Оборудование +16% — базовая инфляция по «железу».</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>КИПиА выросли кратно — не цена, а резко расширенный объём (509 приборов против укрупнённых категорий 2024).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Рекомендация: «CAPEX-2026» = структура ТЭО-2024 + цены 2026 + расценка электрики → итог заметно выше $40,7 млн.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A12:E12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>